<commit_message>
Atualiza template residencial (remove cobertura vazada do empresarial)
O dono do produto enviou o template residencial corrigido: a coluna
"Vendaval, Furacão, Ciclone, Tornado, Granizo e Impacto de Veículos -
para Bens Ao Ar Livre" foi removida — era uma cobertura exclusiva do
empresarial que tinha vazado por engano no template residencial
(mesmo tipo de defeito da coluna "Benefícios Essenciais" vazada no
sentido contrário). Residencial passa de 54 para 53 colunas e de 31
para 30 coberturas.

Também corrige um erro de transcrição em normas_residencial.md: o
teto de R$150.000 e a restrição de UF para vendaval citavam por
engano o nome da cobertura removida, quando a norma de origem sempre
se referiu à cobertura que continua existindo ("...e Fumaça para Bens
Ao Ar Livre").
</commit_message>
<xml_diff>
--- a/templates/template_residencial.xlsx
+++ b/templates/template_residencial.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="90">
   <si>
     <t>Dados CORRETOR</t>
   </si>
@@ -107,9 +107,6 @@
   </si>
   <si>
     <t>TXT "Vendaval, Furacão, Ciclone, Tornado, Granizo, Neve e Geada" Valor da Cobertura</t>
-  </si>
-  <si>
-    <t>TXT "Vendaval, Furacão, Ciclone, Tornado, Granizo e Impacto de Veículos - para Bens Ao Ar Livre" Valor da Cobertura</t>
   </si>
   <si>
     <t>TXT "Roubo E/ou Furto Qualificado de Bens" Valor da Cobertura</t>
@@ -406,12 +403,12 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
@@ -420,10 +417,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="7" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left"/>
@@ -444,9 +441,6 @@
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
@@ -717,8 +711,7 @@
     <col customWidth="1" min="51" max="51" width="60.86"/>
     <col customWidth="1" min="52" max="52" width="94.86"/>
     <col customWidth="1" min="53" max="53" width="87.71"/>
-    <col customWidth="1" min="54" max="54" width="51.43"/>
-    <col customWidth="1" min="55" max="73" width="8.71"/>
+    <col customWidth="1" min="54" max="72" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -740,6 +733,7 @@
       <c r="X1" s="6" t="s">
         <v>5</v>
       </c>
+      <c r="BB1" s="7"/>
       <c r="BC1" s="7"/>
       <c r="BD1" s="7"/>
       <c r="BE1" s="7"/>
@@ -758,7 +752,6 @@
       <c r="BR1" s="7"/>
       <c r="BS1" s="7"/>
       <c r="BT1" s="7"/>
-      <c r="BU1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
@@ -920,173 +913,168 @@
       <c r="BA2" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="BB2" s="10" t="s">
-        <v>59</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>60</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>61</v>
       </c>
       <c r="C3" s="11">
         <v>641755.0</v>
       </c>
       <c r="D3" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="F3" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="G3" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="G3" s="12" t="s">
-        <v>65</v>
-      </c>
       <c r="H3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="M3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="O3" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="I3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="J3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="K3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="L3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="M3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="N3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="O3" s="11" t="s">
+      <c r="P3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="R3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="S3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="T3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="U3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="V3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="W3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="X3" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y3" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="P3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="R3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="S3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="T3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="U3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="V3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="W3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="X3" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y3" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="Z3" s="14" t="s">
-        <v>66</v>
+      <c r="Z3" s="11" t="s">
+        <v>65</v>
       </c>
       <c r="AA3" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AB3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AC3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AD3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AE3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AF3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AH3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AI3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AJ3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AK3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AL3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AM3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AN3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AO3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AP3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AQ3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AR3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AS3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AT3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AU3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AV3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AW3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AX3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AY3" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AZ3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="BA3" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BB3" s="11" t="s">
-        <v>66</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="BB3" s="11"/>
       <c r="BC3" s="11"/>
       <c r="BD3" s="11"/>
       <c r="BE3" s="11"/>
@@ -1105,1318 +1093,1293 @@
       <c r="BR3" s="11"/>
       <c r="BS3" s="11"/>
       <c r="BT3" s="11"/>
-      <c r="BU3" s="11"/>
     </row>
     <row r="4">
       <c r="A4" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>69</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>70</v>
       </c>
       <c r="C4" s="11">
         <v>641755.0</v>
       </c>
       <c r="D4" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="F4" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="G4" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>74</v>
-      </c>
       <c r="H4" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N4" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="O4" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="P4" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="Q4" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="R4" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="S4" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="L4" s="13" t="s">
+      <c r="T4" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="M4" s="13" t="s">
+      <c r="U4" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="N4" s="13" t="s">
+      <c r="V4" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="O4" s="13" t="s">
+      <c r="W4" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="P4" s="11" t="s">
+      <c r="X4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y4" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="Q4" s="11" t="s">
+      <c r="Z4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA4" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="R4" s="11" t="s">
+      <c r="AB4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AM4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AN4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AO4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AP4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AQ4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AR4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AT4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AU4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AV4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AW4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AX4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AY4" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="S4" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="T4" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="U4" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="V4" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="W4" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="X4" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y4" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="Z4" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA4" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="AB4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AE4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AF4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AG4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AH4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AI4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AJ4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AK4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AL4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AM4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AN4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AP4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AQ4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AR4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AS4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AT4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AU4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AV4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AW4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AX4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AY4" s="11" t="s">
-        <v>68</v>
-      </c>
       <c r="AZ4" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="BA4" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BB4" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>75</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>76</v>
       </c>
       <c r="C5" s="11">
         <v>641755.0</v>
       </c>
       <c r="D5" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="F5" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="G5" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="H5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="K5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="M5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="O5" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="P5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="R5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="S5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="T5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="U5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="V5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="W5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="X5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y5" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA5" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AM5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AN5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AO5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AP5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AQ5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AR5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AT5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AU5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AV5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AW5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AX5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AY5" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="AZ5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="BA5" s="11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="B6" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="K6" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="M6" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N6" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="O6" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="P6" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="Q6" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="J5" s="13" t="s">
+      <c r="R6" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="S6" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="L5" s="13" t="s">
+      <c r="T6" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="M5" s="13" t="s">
+      <c r="U6" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="N5" s="13" t="s">
+      <c r="V6" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="O5" s="11" t="s">
+      <c r="W6" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="X6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y6" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="P5" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q5" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="R5" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="S5" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="T5" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="U5" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="V5" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="W5" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="X5" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y5" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="Z5" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA5" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="AB5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AE5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AF5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AG5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AH5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AI5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AJ5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AK5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AL5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AM5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AN5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AP5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AQ5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AR5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AS5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AT5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AU5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AV5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AW5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AX5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AY5" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="AZ5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BA5" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BB5" s="11" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="J6" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="K6" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="L6" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="M6" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="N6" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="O6" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="P6" s="11" t="s">
+      <c r="Z6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA6" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="Q6" s="11" t="s">
+      <c r="AB6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AM6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AN6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AO6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AP6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AQ6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AR6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AT6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AU6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AV6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AW6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AX6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AY6" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="R6" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="S6" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="T6" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="U6" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="V6" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="W6" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="X6" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y6" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="Z6" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA6" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="AB6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AE6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AF6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AG6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AH6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AI6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AJ6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AK6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AL6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AM6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AN6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AP6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AQ6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AR6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AS6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AT6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AU6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AV6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AW6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AX6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AY6" s="11" t="s">
-        <v>68</v>
-      </c>
       <c r="AZ6" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="BA6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BB6" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="B7" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C7" s="11" t="s">
-        <v>83</v>
-      </c>
       <c r="D7" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="K7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="M7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="O7" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="I7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="J7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="K7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="L7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="M7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="N7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="O7" s="11" t="s">
+      <c r="P7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="R7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="S7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="T7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="U7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="V7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="W7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="X7" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y7" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="P7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="R7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="S7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="T7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="U7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="V7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="W7" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="X7" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y7" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="Z7" s="14" t="s">
-        <v>66</v>
+      <c r="Z7" s="11" t="s">
+        <v>65</v>
       </c>
       <c r="AA7" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AB7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AC7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AD7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AE7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AF7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AH7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AI7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AJ7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AK7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AL7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AM7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AN7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AO7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AP7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AQ7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AR7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AS7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AT7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AU7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AV7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AW7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AX7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AY7" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AZ7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="BA7" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BB7" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>83</v>
-      </c>
       <c r="D8" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E8" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F8" s="11" t="s">
-        <v>79</v>
-      </c>
       <c r="G8" s="12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H8" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="K8" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L8" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="M8" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N8" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="O8" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="P8" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="Q8" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="J8" s="13" t="s">
+      <c r="R8" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="S8" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="L8" s="13" t="s">
+      <c r="T8" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="M8" s="13" t="s">
+      <c r="U8" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="N8" s="13" t="s">
+      <c r="V8" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="O8" s="13" t="s">
+      <c r="W8" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="P8" s="11" t="s">
+      <c r="X8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y8" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="Q8" s="11" t="s">
+      <c r="Z8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA8" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="R8" s="11" t="s">
+      <c r="AB8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AM8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AN8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AO8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AP8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AQ8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AR8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AT8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AU8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AV8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AW8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AX8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AY8" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="S8" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="T8" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="U8" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="V8" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="W8" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="X8" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y8" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="Z8" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA8" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="AB8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AE8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AF8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AG8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AH8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AI8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AJ8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AK8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AL8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AM8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AN8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AP8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AQ8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AR8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AS8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AT8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AU8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AV8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AW8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AX8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AY8" s="11" t="s">
-        <v>68</v>
-      </c>
       <c r="AZ8" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="BA8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BB8" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="B9" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>83</v>
-      </c>
       <c r="D9" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="K9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="M9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="O9" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="P9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="R9" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="S9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="T9" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="U9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="V9" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="W9" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="X9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y9" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA9" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AM9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AN9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AO9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AP9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AQ9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AR9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AT9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AU9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AV9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AW9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AX9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AY9" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="AZ9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="BA9" s="11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="E9" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="F9" s="11" t="s">
+      <c r="E10" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="H10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="J10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="K10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="M10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="O10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="P10" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q10" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="R10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="S10" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="T10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="U10" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="V10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="W10" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="X10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y10" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA10" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AM10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AN10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AO10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AP10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AQ10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AR10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AT10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AU10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AV10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AW10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AX10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AY10" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="AZ10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="BA10" s="11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="G11" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="G9" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="H9" s="13" t="s">
+      <c r="H11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="J11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="K11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="M11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="O11" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="P11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="R11" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="S11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="T11" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="U11" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="V11" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="L9" s="13" t="s">
+      <c r="W11" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="M9" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="N9" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="O9" s="11" t="s">
+      <c r="X11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y11" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="P9" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q9" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="R9" s="11" t="s">
+      <c r="Z11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA11" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="S9" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="T9" s="11" t="s">
+      <c r="AB11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AM11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AN11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AO11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AP11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AQ11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AR11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AT11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AU11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AV11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AW11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AX11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AY11" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="U9" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="V9" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="W9" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="X9" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y9" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="Z9" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA9" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="AB9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AE9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AF9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AG9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AH9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AI9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AJ9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AK9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AL9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AM9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AN9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AP9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AQ9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AR9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AS9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AT9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AU9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AV9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AW9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AX9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AY9" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="AZ9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BA9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BB9" s="11" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="H10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="I10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="J10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="K10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="L10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="M10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="N10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="O10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="P10" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q10" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="R10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="S10" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="T10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="U10" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="V10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="W10" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="X10" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y10" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="Z10" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA10" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="AB10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AE10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AF10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AG10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AH10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AI10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AJ10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AK10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AL10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AM10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AN10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AP10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AQ10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AR10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AS10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AT10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AU10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AV10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AW10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AX10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AY10" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="AZ10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BA10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BB10" s="11" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="H11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="I11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="J11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="K11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="L11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="M11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="N11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="O11" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="P11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="R11" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="S11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="T11" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="U11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="V11" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="W11" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="X11" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y11" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="Z11" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA11" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="AB11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AE11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AF11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AG11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AH11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AI11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AJ11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AK11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AL11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AM11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AN11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AO11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AP11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AQ11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AR11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AS11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AT11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AU11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AV11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AW11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AX11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AY11" s="11" t="s">
-        <v>68</v>
-      </c>
       <c r="AZ11" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="BA11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="BB11" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12">
@@ -2470,7 +2433,6 @@
       <c r="AY12" s="11"/>
       <c r="AZ12" s="11"/>
       <c r="BA12" s="11"/>
-      <c r="BB12" s="11"/>
     </row>
     <row r="13">
       <c r="D13" s="11"/>
@@ -2523,7 +2485,6 @@
       <c r="AY13" s="11"/>
       <c r="AZ13" s="11"/>
       <c r="BA13" s="11"/>
-      <c r="BB13" s="11"/>
     </row>
     <row r="14">
       <c r="D14" s="11"/>
@@ -2576,7 +2537,6 @@
       <c r="AY14" s="11"/>
       <c r="AZ14" s="11"/>
       <c r="BA14" s="11"/>
-      <c r="BB14" s="11"/>
     </row>
     <row r="15">
       <c r="D15" s="11"/>
@@ -2629,7 +2589,6 @@
       <c r="AY15" s="11"/>
       <c r="AZ15" s="11"/>
       <c r="BA15" s="11"/>
-      <c r="BB15" s="11"/>
     </row>
     <row r="16">
       <c r="D16" s="11"/>
@@ -2682,7 +2641,6 @@
       <c r="AY16" s="11"/>
       <c r="AZ16" s="11"/>
       <c r="BA16" s="11"/>
-      <c r="BB16" s="11"/>
     </row>
     <row r="17">
       <c r="D17" s="11"/>
@@ -2735,7 +2693,6 @@
       <c r="AY17" s="11"/>
       <c r="AZ17" s="11"/>
       <c r="BA17" s="11"/>
-      <c r="BB17" s="11"/>
     </row>
     <row r="18">
       <c r="D18" s="11"/>
@@ -2788,7 +2745,6 @@
       <c r="AY18" s="11"/>
       <c r="AZ18" s="11"/>
       <c r="BA18" s="11"/>
-      <c r="BB18" s="11"/>
     </row>
     <row r="19">
       <c r="D19" s="11"/>
@@ -2841,7 +2797,6 @@
       <c r="AY19" s="11"/>
       <c r="AZ19" s="11"/>
       <c r="BA19" s="11"/>
-      <c r="BB19" s="11"/>
     </row>
     <row r="20">
       <c r="D20" s="11"/>
@@ -2894,7 +2849,6 @@
       <c r="AY20" s="11"/>
       <c r="AZ20" s="11"/>
       <c r="BA20" s="11"/>
-      <c r="BB20" s="11"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="D21" s="11"/>
@@ -2947,7 +2901,6 @@
       <c r="AY21" s="11"/>
       <c r="AZ21" s="11"/>
       <c r="BA21" s="11"/>
-      <c r="BB21" s="11"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="D22" s="11"/>
@@ -3000,7 +2953,6 @@
       <c r="AY22" s="11"/>
       <c r="AZ22" s="11"/>
       <c r="BA22" s="11"/>
-      <c r="BB22" s="11"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="D23" s="11"/>
@@ -3053,7 +3005,6 @@
       <c r="AY23" s="11"/>
       <c r="AZ23" s="11"/>
       <c r="BA23" s="11"/>
-      <c r="BB23" s="11"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="D24" s="11"/>
@@ -3106,7 +3057,6 @@
       <c r="AY24" s="11"/>
       <c r="AZ24" s="11"/>
       <c r="BA24" s="11"/>
-      <c r="BB24" s="11"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="D25" s="11"/>
@@ -3159,7 +3109,6 @@
       <c r="AY25" s="11"/>
       <c r="AZ25" s="11"/>
       <c r="BA25" s="11"/>
-      <c r="BB25" s="11"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="D26" s="11"/>
@@ -3212,7 +3161,6 @@
       <c r="AY26" s="11"/>
       <c r="AZ26" s="11"/>
       <c r="BA26" s="11"/>
-      <c r="BB26" s="11"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="D27" s="11"/>
@@ -3265,7 +3213,6 @@
       <c r="AY27" s="11"/>
       <c r="AZ27" s="11"/>
       <c r="BA27" s="11"/>
-      <c r="BB27" s="11"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="D28" s="11"/>
@@ -3318,7 +3265,6 @@
       <c r="AY28" s="11"/>
       <c r="AZ28" s="11"/>
       <c r="BA28" s="11"/>
-      <c r="BB28" s="11"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="D29" s="11"/>
@@ -3371,7 +3317,6 @@
       <c r="AY29" s="11"/>
       <c r="AZ29" s="11"/>
       <c r="BA29" s="11"/>
-      <c r="BB29" s="11"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="D30" s="11"/>
@@ -3424,7 +3369,6 @@
       <c r="AY30" s="11"/>
       <c r="AZ30" s="11"/>
       <c r="BA30" s="11"/>
-      <c r="BB30" s="11"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="D31" s="11"/>
@@ -3477,7 +3421,6 @@
       <c r="AY31" s="11"/>
       <c r="AZ31" s="11"/>
       <c r="BA31" s="11"/>
-      <c r="BB31" s="11"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="D32" s="11"/>
@@ -3530,7 +3473,6 @@
       <c r="AY32" s="11"/>
       <c r="AZ32" s="11"/>
       <c r="BA32" s="11"/>
-      <c r="BB32" s="11"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="D33" s="11"/>
@@ -3583,7 +3525,6 @@
       <c r="AY33" s="11"/>
       <c r="AZ33" s="11"/>
       <c r="BA33" s="11"/>
-      <c r="BB33" s="11"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="D34" s="11"/>
@@ -3636,7 +3577,6 @@
       <c r="AY34" s="11"/>
       <c r="AZ34" s="11"/>
       <c r="BA34" s="11"/>
-      <c r="BB34" s="11"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="D35" s="11"/>
@@ -3689,7 +3629,6 @@
       <c r="AY35" s="11"/>
       <c r="AZ35" s="11"/>
       <c r="BA35" s="11"/>
-      <c r="BB35" s="11"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="D36" s="11"/>
@@ -3742,7 +3681,6 @@
       <c r="AY36" s="11"/>
       <c r="AZ36" s="11"/>
       <c r="BA36" s="11"/>
-      <c r="BB36" s="11"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="D37" s="11"/>
@@ -3795,7 +3733,6 @@
       <c r="AY37" s="11"/>
       <c r="AZ37" s="11"/>
       <c r="BA37" s="11"/>
-      <c r="BB37" s="11"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="D38" s="11"/>
@@ -3848,7 +3785,6 @@
       <c r="AY38" s="11"/>
       <c r="AZ38" s="11"/>
       <c r="BA38" s="11"/>
-      <c r="BB38" s="11"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="D39" s="11"/>
@@ -3901,7 +3837,6 @@
       <c r="AY39" s="11"/>
       <c r="AZ39" s="11"/>
       <c r="BA39" s="11"/>
-      <c r="BB39" s="11"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="D40" s="11"/>
@@ -3954,7 +3889,6 @@
       <c r="AY40" s="11"/>
       <c r="AZ40" s="11"/>
       <c r="BA40" s="11"/>
-      <c r="BB40" s="11"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="D41" s="11"/>
@@ -4007,7 +3941,6 @@
       <c r="AY41" s="11"/>
       <c r="AZ41" s="11"/>
       <c r="BA41" s="11"/>
-      <c r="BB41" s="11"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="D42" s="11"/>
@@ -4060,7 +3993,6 @@
       <c r="AY42" s="11"/>
       <c r="AZ42" s="11"/>
       <c r="BA42" s="11"/>
-      <c r="BB42" s="11"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="D43" s="11"/>
@@ -4113,7 +4045,6 @@
       <c r="AY43" s="11"/>
       <c r="AZ43" s="11"/>
       <c r="BA43" s="11"/>
-      <c r="BB43" s="11"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="D44" s="11"/>
@@ -4166,7 +4097,6 @@
       <c r="AY44" s="11"/>
       <c r="AZ44" s="11"/>
       <c r="BA44" s="11"/>
-      <c r="BB44" s="11"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="D45" s="11"/>
@@ -4219,7 +4149,6 @@
       <c r="AY45" s="11"/>
       <c r="AZ45" s="11"/>
       <c r="BA45" s="11"/>
-      <c r="BB45" s="11"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="D46" s="11"/>
@@ -4272,7 +4201,6 @@
       <c r="AY46" s="11"/>
       <c r="AZ46" s="11"/>
       <c r="BA46" s="11"/>
-      <c r="BB46" s="11"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="D47" s="11"/>
@@ -4325,7 +4253,6 @@
       <c r="AY47" s="11"/>
       <c r="AZ47" s="11"/>
       <c r="BA47" s="11"/>
-      <c r="BB47" s="11"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="D48" s="11"/>
@@ -4378,7 +4305,6 @@
       <c r="AY48" s="11"/>
       <c r="AZ48" s="11"/>
       <c r="BA48" s="11"/>
-      <c r="BB48" s="11"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="D49" s="11"/>
@@ -4431,7 +4357,6 @@
       <c r="AY49" s="11"/>
       <c r="AZ49" s="11"/>
       <c r="BA49" s="11"/>
-      <c r="BB49" s="11"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="D50" s="11"/>
@@ -4484,7 +4409,6 @@
       <c r="AY50" s="11"/>
       <c r="AZ50" s="11"/>
       <c r="BA50" s="11"/>
-      <c r="BB50" s="11"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="D51" s="11"/>
@@ -4537,7 +4461,6 @@
       <c r="AY51" s="11"/>
       <c r="AZ51" s="11"/>
       <c r="BA51" s="11"/>
-      <c r="BB51" s="11"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="D52" s="11"/>
@@ -4590,7 +4513,6 @@
       <c r="AY52" s="11"/>
       <c r="AZ52" s="11"/>
       <c r="BA52" s="11"/>
-      <c r="BB52" s="11"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="D53" s="11"/>
@@ -4643,7 +4565,6 @@
       <c r="AY53" s="11"/>
       <c r="AZ53" s="11"/>
       <c r="BA53" s="11"/>
-      <c r="BB53" s="11"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="D54" s="11"/>
@@ -4696,7 +4617,6 @@
       <c r="AY54" s="11"/>
       <c r="AZ54" s="11"/>
       <c r="BA54" s="11"/>
-      <c r="BB54" s="11"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="D55" s="11"/>
@@ -4749,7 +4669,6 @@
       <c r="AY55" s="11"/>
       <c r="AZ55" s="11"/>
       <c r="BA55" s="11"/>
-      <c r="BB55" s="11"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="D56" s="11"/>
@@ -4802,7 +4721,6 @@
       <c r="AY56" s="11"/>
       <c r="AZ56" s="11"/>
       <c r="BA56" s="11"/>
-      <c r="BB56" s="11"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="D57" s="11"/>
@@ -4855,7 +4773,6 @@
       <c r="AY57" s="11"/>
       <c r="AZ57" s="11"/>
       <c r="BA57" s="11"/>
-      <c r="BB57" s="11"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="D58" s="11"/>
@@ -4908,7 +4825,6 @@
       <c r="AY58" s="11"/>
       <c r="AZ58" s="11"/>
       <c r="BA58" s="11"/>
-      <c r="BB58" s="11"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="D59" s="11"/>
@@ -4961,7 +4877,6 @@
       <c r="AY59" s="11"/>
       <c r="AZ59" s="11"/>
       <c r="BA59" s="11"/>
-      <c r="BB59" s="11"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="D60" s="11"/>
@@ -5014,7 +4929,6 @@
       <c r="AY60" s="11"/>
       <c r="AZ60" s="11"/>
       <c r="BA60" s="11"/>
-      <c r="BB60" s="11"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="D61" s="11"/>
@@ -5067,7 +4981,6 @@
       <c r="AY61" s="11"/>
       <c r="AZ61" s="11"/>
       <c r="BA61" s="11"/>
-      <c r="BB61" s="11"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="D62" s="11"/>
@@ -5120,7 +5033,6 @@
       <c r="AY62" s="11"/>
       <c r="AZ62" s="11"/>
       <c r="BA62" s="11"/>
-      <c r="BB62" s="11"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="D63" s="11"/>
@@ -5173,7 +5085,6 @@
       <c r="AY63" s="11"/>
       <c r="AZ63" s="11"/>
       <c r="BA63" s="11"/>
-      <c r="BB63" s="11"/>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="D64" s="11"/>
@@ -5226,7 +5137,6 @@
       <c r="AY64" s="11"/>
       <c r="AZ64" s="11"/>
       <c r="BA64" s="11"/>
-      <c r="BB64" s="11"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="D65" s="11"/>
@@ -5279,7 +5189,6 @@
       <c r="AY65" s="11"/>
       <c r="AZ65" s="11"/>
       <c r="BA65" s="11"/>
-      <c r="BB65" s="11"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="D66" s="11"/>
@@ -5332,7 +5241,6 @@
       <c r="AY66" s="11"/>
       <c r="AZ66" s="11"/>
       <c r="BA66" s="11"/>
-      <c r="BB66" s="11"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="D67" s="11"/>
@@ -5385,7 +5293,6 @@
       <c r="AY67" s="11"/>
       <c r="AZ67" s="11"/>
       <c r="BA67" s="11"/>
-      <c r="BB67" s="11"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="D68" s="11"/>
@@ -5438,7 +5345,6 @@
       <c r="AY68" s="11"/>
       <c r="AZ68" s="11"/>
       <c r="BA68" s="11"/>
-      <c r="BB68" s="11"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="D69" s="11"/>
@@ -5491,7 +5397,6 @@
       <c r="AY69" s="11"/>
       <c r="AZ69" s="11"/>
       <c r="BA69" s="11"/>
-      <c r="BB69" s="11"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="D70" s="11"/>
@@ -5544,7 +5449,6 @@
       <c r="AY70" s="11"/>
       <c r="AZ70" s="11"/>
       <c r="BA70" s="11"/>
-      <c r="BB70" s="11"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="D71" s="11"/>
@@ -5597,7 +5501,6 @@
       <c r="AY71" s="11"/>
       <c r="AZ71" s="11"/>
       <c r="BA71" s="11"/>
-      <c r="BB71" s="11"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="D72" s="11"/>
@@ -5650,7 +5553,6 @@
       <c r="AY72" s="11"/>
       <c r="AZ72" s="11"/>
       <c r="BA72" s="11"/>
-      <c r="BB72" s="11"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="D73" s="11"/>
@@ -5703,7 +5605,6 @@
       <c r="AY73" s="11"/>
       <c r="AZ73" s="11"/>
       <c r="BA73" s="11"/>
-      <c r="BB73" s="11"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="D74" s="11"/>
@@ -5756,7 +5657,6 @@
       <c r="AY74" s="11"/>
       <c r="AZ74" s="11"/>
       <c r="BA74" s="11"/>
-      <c r="BB74" s="11"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="D75" s="11"/>
@@ -5809,7 +5709,6 @@
       <c r="AY75" s="11"/>
       <c r="AZ75" s="11"/>
       <c r="BA75" s="11"/>
-      <c r="BB75" s="11"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="D76" s="11"/>
@@ -5862,7 +5761,6 @@
       <c r="AY76" s="11"/>
       <c r="AZ76" s="11"/>
       <c r="BA76" s="11"/>
-      <c r="BB76" s="11"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="D77" s="11"/>
@@ -5915,7 +5813,6 @@
       <c r="AY77" s="11"/>
       <c r="AZ77" s="11"/>
       <c r="BA77" s="11"/>
-      <c r="BB77" s="11"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
       <c r="D78" s="11"/>
@@ -5968,7 +5865,6 @@
       <c r="AY78" s="11"/>
       <c r="AZ78" s="11"/>
       <c r="BA78" s="11"/>
-      <c r="BB78" s="11"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="D79" s="11"/>
@@ -6021,7 +5917,6 @@
       <c r="AY79" s="11"/>
       <c r="AZ79" s="11"/>
       <c r="BA79" s="11"/>
-      <c r="BB79" s="11"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="D80" s="11"/>
@@ -6074,7 +5969,6 @@
       <c r="AY80" s="11"/>
       <c r="AZ80" s="11"/>
       <c r="BA80" s="11"/>
-      <c r="BB80" s="11"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="D81" s="11"/>
@@ -6127,7 +6021,6 @@
       <c r="AY81" s="11"/>
       <c r="AZ81" s="11"/>
       <c r="BA81" s="11"/>
-      <c r="BB81" s="11"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="D82" s="11"/>
@@ -6180,7 +6073,6 @@
       <c r="AY82" s="11"/>
       <c r="AZ82" s="11"/>
       <c r="BA82" s="11"/>
-      <c r="BB82" s="11"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="D83" s="11"/>
@@ -6233,7 +6125,6 @@
       <c r="AY83" s="11"/>
       <c r="AZ83" s="11"/>
       <c r="BA83" s="11"/>
-      <c r="BB83" s="11"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="D84" s="11"/>
@@ -6286,7 +6177,6 @@
       <c r="AY84" s="11"/>
       <c r="AZ84" s="11"/>
       <c r="BA84" s="11"/>
-      <c r="BB84" s="11"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="D85" s="11"/>
@@ -6339,7 +6229,6 @@
       <c r="AY85" s="11"/>
       <c r="AZ85" s="11"/>
       <c r="BA85" s="11"/>
-      <c r="BB85" s="11"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
       <c r="D86" s="11"/>
@@ -6392,7 +6281,6 @@
       <c r="AY86" s="11"/>
       <c r="AZ86" s="11"/>
       <c r="BA86" s="11"/>
-      <c r="BB86" s="11"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="D87" s="11"/>
@@ -6445,7 +6333,6 @@
       <c r="AY87" s="11"/>
       <c r="AZ87" s="11"/>
       <c r="BA87" s="11"/>
-      <c r="BB87" s="11"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
       <c r="D88" s="11"/>
@@ -6498,7 +6385,6 @@
       <c r="AY88" s="11"/>
       <c r="AZ88" s="11"/>
       <c r="BA88" s="11"/>
-      <c r="BB88" s="11"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="D89" s="11"/>
@@ -6551,7 +6437,6 @@
       <c r="AY89" s="11"/>
       <c r="AZ89" s="11"/>
       <c r="BA89" s="11"/>
-      <c r="BB89" s="11"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="D90" s="11"/>
@@ -6604,7 +6489,6 @@
       <c r="AY90" s="11"/>
       <c r="AZ90" s="11"/>
       <c r="BA90" s="11"/>
-      <c r="BB90" s="11"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="D91" s="11"/>
@@ -6657,7 +6541,6 @@
       <c r="AY91" s="11"/>
       <c r="AZ91" s="11"/>
       <c r="BA91" s="11"/>
-      <c r="BB91" s="11"/>
     </row>
     <row r="92" ht="15.75" customHeight="1">
       <c r="D92" s="11"/>
@@ -6710,7 +6593,6 @@
       <c r="AY92" s="11"/>
       <c r="AZ92" s="11"/>
       <c r="BA92" s="11"/>
-      <c r="BB92" s="11"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
       <c r="D93" s="11"/>
@@ -6763,7 +6645,6 @@
       <c r="AY93" s="11"/>
       <c r="AZ93" s="11"/>
       <c r="BA93" s="11"/>
-      <c r="BB93" s="11"/>
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="D94" s="11"/>
@@ -6816,7 +6697,6 @@
       <c r="AY94" s="11"/>
       <c r="AZ94" s="11"/>
       <c r="BA94" s="11"/>
-      <c r="BB94" s="11"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="D95" s="11"/>
@@ -6869,7 +6749,6 @@
       <c r="AY95" s="11"/>
       <c r="AZ95" s="11"/>
       <c r="BA95" s="11"/>
-      <c r="BB95" s="11"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="D96" s="11"/>
@@ -6922,7 +6801,6 @@
       <c r="AY96" s="11"/>
       <c r="AZ96" s="11"/>
       <c r="BA96" s="11"/>
-      <c r="BB96" s="11"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="D97" s="11"/>
@@ -6975,7 +6853,6 @@
       <c r="AY97" s="11"/>
       <c r="AZ97" s="11"/>
       <c r="BA97" s="11"/>
-      <c r="BB97" s="11"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="D98" s="11"/>
@@ -7028,7 +6905,6 @@
       <c r="AY98" s="11"/>
       <c r="AZ98" s="11"/>
       <c r="BA98" s="11"/>
-      <c r="BB98" s="11"/>
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="D99" s="11"/>
@@ -7081,7 +6957,6 @@
       <c r="AY99" s="11"/>
       <c r="AZ99" s="11"/>
       <c r="BA99" s="11"/>
-      <c r="BB99" s="11"/>
     </row>
     <row r="100" ht="15.75" customHeight="1">
       <c r="D100" s="11"/>
@@ -7134,7 +7009,6 @@
       <c r="AY100" s="11"/>
       <c r="AZ100" s="11"/>
       <c r="BA100" s="11"/>
-      <c r="BB100" s="11"/>
     </row>
     <row r="101" ht="15.75" customHeight="1">
       <c r="D101" s="11"/>
@@ -7187,7 +7061,6 @@
       <c r="AY101" s="11"/>
       <c r="AZ101" s="11"/>
       <c r="BA101" s="11"/>
-      <c r="BB101" s="11"/>
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="D102" s="11"/>
@@ -7240,7 +7113,6 @@
       <c r="AY102" s="11"/>
       <c r="AZ102" s="11"/>
       <c r="BA102" s="11"/>
-      <c r="BB102" s="11"/>
     </row>
     <row r="103" ht="15.75" customHeight="1">
       <c r="D103" s="11"/>
@@ -7293,7 +7165,6 @@
       <c r="AY103" s="11"/>
       <c r="AZ103" s="11"/>
       <c r="BA103" s="11"/>
-      <c r="BB103" s="11"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
       <c r="D104" s="11"/>
@@ -7346,7 +7217,6 @@
       <c r="AY104" s="11"/>
       <c r="AZ104" s="11"/>
       <c r="BA104" s="11"/>
-      <c r="BB104" s="11"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
       <c r="D105" s="11"/>
@@ -7399,7 +7269,6 @@
       <c r="AY105" s="11"/>
       <c r="AZ105" s="11"/>
       <c r="BA105" s="11"/>
-      <c r="BB105" s="11"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
       <c r="D106" s="11"/>
@@ -7452,7 +7321,6 @@
       <c r="AY106" s="11"/>
       <c r="AZ106" s="11"/>
       <c r="BA106" s="11"/>
-      <c r="BB106" s="11"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
       <c r="D107" s="11"/>
@@ -7505,7 +7373,6 @@
       <c r="AY107" s="11"/>
       <c r="AZ107" s="11"/>
       <c r="BA107" s="11"/>
-      <c r="BB107" s="11"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
       <c r="D108" s="11"/>
@@ -7558,7 +7425,6 @@
       <c r="AY108" s="11"/>
       <c r="AZ108" s="11"/>
       <c r="BA108" s="11"/>
-      <c r="BB108" s="11"/>
     </row>
     <row r="109" ht="15.75" customHeight="1">
       <c r="D109" s="11"/>
@@ -7611,7 +7477,6 @@
       <c r="AY109" s="11"/>
       <c r="AZ109" s="11"/>
       <c r="BA109" s="11"/>
-      <c r="BB109" s="11"/>
     </row>
     <row r="110" ht="15.75" customHeight="1">
       <c r="D110" s="11"/>
@@ -7664,7 +7529,6 @@
       <c r="AY110" s="11"/>
       <c r="AZ110" s="11"/>
       <c r="BA110" s="11"/>
-      <c r="BB110" s="11"/>
     </row>
     <row r="111" ht="15.75" customHeight="1">
       <c r="D111" s="11"/>
@@ -7717,7 +7581,6 @@
       <c r="AY111" s="11"/>
       <c r="AZ111" s="11"/>
       <c r="BA111" s="11"/>
-      <c r="BB111" s="11"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
       <c r="D112" s="11"/>
@@ -7770,7 +7633,6 @@
       <c r="AY112" s="11"/>
       <c r="AZ112" s="11"/>
       <c r="BA112" s="11"/>
-      <c r="BB112" s="11"/>
     </row>
     <row r="113" ht="15.75" customHeight="1">
       <c r="D113" s="11"/>
@@ -7823,7 +7685,6 @@
       <c r="AY113" s="11"/>
       <c r="AZ113" s="11"/>
       <c r="BA113" s="11"/>
-      <c r="BB113" s="11"/>
     </row>
     <row r="114" ht="15.75" customHeight="1">
       <c r="D114" s="11"/>
@@ -7876,7 +7737,6 @@
       <c r="AY114" s="11"/>
       <c r="AZ114" s="11"/>
       <c r="BA114" s="11"/>
-      <c r="BB114" s="11"/>
     </row>
     <row r="115" ht="15.75" customHeight="1">
       <c r="D115" s="11"/>
@@ -7929,7 +7789,6 @@
       <c r="AY115" s="11"/>
       <c r="AZ115" s="11"/>
       <c r="BA115" s="11"/>
-      <c r="BB115" s="11"/>
     </row>
     <row r="116" ht="15.75" customHeight="1">
       <c r="D116" s="11"/>
@@ -7982,7 +7841,6 @@
       <c r="AY116" s="11"/>
       <c r="AZ116" s="11"/>
       <c r="BA116" s="11"/>
-      <c r="BB116" s="11"/>
     </row>
     <row r="117" ht="15.75" customHeight="1">
       <c r="D117" s="11"/>
@@ -8035,7 +7893,6 @@
       <c r="AY117" s="11"/>
       <c r="AZ117" s="11"/>
       <c r="BA117" s="11"/>
-      <c r="BB117" s="11"/>
     </row>
     <row r="118" ht="15.75" customHeight="1">
       <c r="D118" s="11"/>
@@ -8088,7 +7945,6 @@
       <c r="AY118" s="11"/>
       <c r="AZ118" s="11"/>
       <c r="BA118" s="11"/>
-      <c r="BB118" s="11"/>
     </row>
     <row r="119" ht="15.75" customHeight="1">
       <c r="D119" s="11"/>
@@ -8141,7 +7997,6 @@
       <c r="AY119" s="11"/>
       <c r="AZ119" s="11"/>
       <c r="BA119" s="11"/>
-      <c r="BB119" s="11"/>
     </row>
     <row r="120" ht="15.75" customHeight="1">
       <c r="D120" s="11"/>
@@ -8194,7 +8049,6 @@
       <c r="AY120" s="11"/>
       <c r="AZ120" s="11"/>
       <c r="BA120" s="11"/>
-      <c r="BB120" s="11"/>
     </row>
     <row r="121" ht="15.75" customHeight="1">
       <c r="D121" s="11"/>
@@ -8247,7 +8101,6 @@
       <c r="AY121" s="11"/>
       <c r="AZ121" s="11"/>
       <c r="BA121" s="11"/>
-      <c r="BB121" s="11"/>
     </row>
     <row r="122" ht="15.75" customHeight="1">
       <c r="D122" s="11"/>
@@ -8300,7 +8153,6 @@
       <c r="AY122" s="11"/>
       <c r="AZ122" s="11"/>
       <c r="BA122" s="11"/>
-      <c r="BB122" s="11"/>
     </row>
     <row r="123" ht="15.75" customHeight="1">
       <c r="D123" s="11"/>
@@ -8353,7 +8205,6 @@
       <c r="AY123" s="11"/>
       <c r="AZ123" s="11"/>
       <c r="BA123" s="11"/>
-      <c r="BB123" s="11"/>
     </row>
     <row r="124" ht="15.75" customHeight="1">
       <c r="D124" s="11"/>
@@ -8406,7 +8257,6 @@
       <c r="AY124" s="11"/>
       <c r="AZ124" s="11"/>
       <c r="BA124" s="11"/>
-      <c r="BB124" s="11"/>
     </row>
     <row r="125" ht="15.75" customHeight="1">
       <c r="D125" s="11"/>
@@ -8459,7 +8309,6 @@
       <c r="AY125" s="11"/>
       <c r="AZ125" s="11"/>
       <c r="BA125" s="11"/>
-      <c r="BB125" s="11"/>
     </row>
     <row r="126" ht="15.75" customHeight="1">
       <c r="D126" s="11"/>
@@ -8512,7 +8361,6 @@
       <c r="AY126" s="11"/>
       <c r="AZ126" s="11"/>
       <c r="BA126" s="11"/>
-      <c r="BB126" s="11"/>
     </row>
     <row r="127" ht="15.75" customHeight="1">
       <c r="D127" s="11"/>
@@ -8565,7 +8413,6 @@
       <c r="AY127" s="11"/>
       <c r="AZ127" s="11"/>
       <c r="BA127" s="11"/>
-      <c r="BB127" s="11"/>
     </row>
     <row r="128" ht="15.75" customHeight="1">
       <c r="D128" s="11"/>
@@ -8618,7 +8465,6 @@
       <c r="AY128" s="11"/>
       <c r="AZ128" s="11"/>
       <c r="BA128" s="11"/>
-      <c r="BB128" s="11"/>
     </row>
     <row r="129" ht="15.75" customHeight="1">
       <c r="D129" s="11"/>
@@ -8671,7 +8517,6 @@
       <c r="AY129" s="11"/>
       <c r="AZ129" s="11"/>
       <c r="BA129" s="11"/>
-      <c r="BB129" s="11"/>
     </row>
     <row r="130" ht="15.75" customHeight="1">
       <c r="D130" s="11"/>
@@ -8724,7 +8569,6 @@
       <c r="AY130" s="11"/>
       <c r="AZ130" s="11"/>
       <c r="BA130" s="11"/>
-      <c r="BB130" s="11"/>
     </row>
     <row r="131" ht="15.75" customHeight="1">
       <c r="D131" s="11"/>
@@ -8777,7 +8621,6 @@
       <c r="AY131" s="11"/>
       <c r="AZ131" s="11"/>
       <c r="BA131" s="11"/>
-      <c r="BB131" s="11"/>
     </row>
     <row r="132" ht="15.75" customHeight="1">
       <c r="D132" s="11"/>
@@ -8830,7 +8673,6 @@
       <c r="AY132" s="11"/>
       <c r="AZ132" s="11"/>
       <c r="BA132" s="11"/>
-      <c r="BB132" s="11"/>
     </row>
     <row r="133" ht="15.75" customHeight="1">
       <c r="D133" s="11"/>
@@ -8883,7 +8725,6 @@
       <c r="AY133" s="11"/>
       <c r="AZ133" s="11"/>
       <c r="BA133" s="11"/>
-      <c r="BB133" s="11"/>
     </row>
     <row r="134" ht="15.75" customHeight="1">
       <c r="D134" s="11"/>
@@ -8936,7 +8777,6 @@
       <c r="AY134" s="11"/>
       <c r="AZ134" s="11"/>
       <c r="BA134" s="11"/>
-      <c r="BB134" s="11"/>
     </row>
     <row r="135" ht="15.75" customHeight="1">
       <c r="D135" s="11"/>
@@ -8989,7 +8829,6 @@
       <c r="AY135" s="11"/>
       <c r="AZ135" s="11"/>
       <c r="BA135" s="11"/>
-      <c r="BB135" s="11"/>
     </row>
     <row r="136" ht="15.75" customHeight="1">
       <c r="D136" s="11"/>
@@ -9042,7 +8881,6 @@
       <c r="AY136" s="11"/>
       <c r="AZ136" s="11"/>
       <c r="BA136" s="11"/>
-      <c r="BB136" s="11"/>
     </row>
     <row r="137" ht="15.75" customHeight="1">
       <c r="D137" s="11"/>
@@ -9095,7 +8933,6 @@
       <c r="AY137" s="11"/>
       <c r="AZ137" s="11"/>
       <c r="BA137" s="11"/>
-      <c r="BB137" s="11"/>
     </row>
     <row r="138" ht="15.75" customHeight="1">
       <c r="D138" s="11"/>
@@ -9148,7 +8985,6 @@
       <c r="AY138" s="11"/>
       <c r="AZ138" s="11"/>
       <c r="BA138" s="11"/>
-      <c r="BB138" s="11"/>
     </row>
     <row r="139" ht="15.75" customHeight="1">
       <c r="D139" s="11"/>
@@ -9201,7 +9037,6 @@
       <c r="AY139" s="11"/>
       <c r="AZ139" s="11"/>
       <c r="BA139" s="11"/>
-      <c r="BB139" s="11"/>
     </row>
     <row r="140" ht="15.75" customHeight="1">
       <c r="D140" s="11"/>
@@ -9254,7 +9089,6 @@
       <c r="AY140" s="11"/>
       <c r="AZ140" s="11"/>
       <c r="BA140" s="11"/>
-      <c r="BB140" s="11"/>
     </row>
     <row r="141" ht="15.75" customHeight="1">
       <c r="D141" s="11"/>
@@ -9307,7 +9141,6 @@
       <c r="AY141" s="11"/>
       <c r="AZ141" s="11"/>
       <c r="BA141" s="11"/>
-      <c r="BB141" s="11"/>
     </row>
     <row r="142" ht="15.75" customHeight="1">
       <c r="D142" s="11"/>
@@ -9360,7 +9193,6 @@
       <c r="AY142" s="11"/>
       <c r="AZ142" s="11"/>
       <c r="BA142" s="11"/>
-      <c r="BB142" s="11"/>
     </row>
     <row r="143" ht="15.75" customHeight="1">
       <c r="D143" s="11"/>
@@ -9413,7 +9245,6 @@
       <c r="AY143" s="11"/>
       <c r="AZ143" s="11"/>
       <c r="BA143" s="11"/>
-      <c r="BB143" s="11"/>
     </row>
     <row r="144" ht="15.75" customHeight="1">
       <c r="D144" s="11"/>
@@ -9466,7 +9297,6 @@
       <c r="AY144" s="11"/>
       <c r="AZ144" s="11"/>
       <c r="BA144" s="11"/>
-      <c r="BB144" s="11"/>
     </row>
     <row r="145" ht="15.75" customHeight="1">
       <c r="D145" s="11"/>
@@ -9519,7 +9349,6 @@
       <c r="AY145" s="11"/>
       <c r="AZ145" s="11"/>
       <c r="BA145" s="11"/>
-      <c r="BB145" s="11"/>
     </row>
     <row r="146" ht="15.75" customHeight="1">
       <c r="D146" s="11"/>
@@ -9572,7 +9401,6 @@
       <c r="AY146" s="11"/>
       <c r="AZ146" s="11"/>
       <c r="BA146" s="11"/>
-      <c r="BB146" s="11"/>
     </row>
     <row r="147" ht="15.75" customHeight="1">
       <c r="D147" s="11"/>
@@ -9625,7 +9453,6 @@
       <c r="AY147" s="11"/>
       <c r="AZ147" s="11"/>
       <c r="BA147" s="11"/>
-      <c r="BB147" s="11"/>
     </row>
     <row r="148" ht="15.75" customHeight="1">
       <c r="D148" s="11"/>
@@ -9678,7 +9505,6 @@
       <c r="AY148" s="11"/>
       <c r="AZ148" s="11"/>
       <c r="BA148" s="11"/>
-      <c r="BB148" s="11"/>
     </row>
     <row r="149" ht="15.75" customHeight="1">
       <c r="D149" s="11"/>
@@ -9731,7 +9557,6 @@
       <c r="AY149" s="11"/>
       <c r="AZ149" s="11"/>
       <c r="BA149" s="11"/>
-      <c r="BB149" s="11"/>
     </row>
     <row r="150" ht="15.75" customHeight="1">
       <c r="D150" s="11"/>
@@ -9784,7 +9609,6 @@
       <c r="AY150" s="11"/>
       <c r="AZ150" s="11"/>
       <c r="BA150" s="11"/>
-      <c r="BB150" s="11"/>
     </row>
     <row r="151" ht="15.75" customHeight="1">
       <c r="D151" s="11"/>
@@ -9837,7 +9661,6 @@
       <c r="AY151" s="11"/>
       <c r="AZ151" s="11"/>
       <c r="BA151" s="11"/>
-      <c r="BB151" s="11"/>
     </row>
     <row r="152" ht="15.75" customHeight="1">
       <c r="D152" s="11"/>
@@ -9890,7 +9713,6 @@
       <c r="AY152" s="11"/>
       <c r="AZ152" s="11"/>
       <c r="BA152" s="11"/>
-      <c r="BB152" s="11"/>
     </row>
     <row r="153" ht="15.75" customHeight="1">
       <c r="D153" s="11"/>
@@ -9943,7 +9765,6 @@
       <c r="AY153" s="11"/>
       <c r="AZ153" s="11"/>
       <c r="BA153" s="11"/>
-      <c r="BB153" s="11"/>
     </row>
     <row r="154" ht="15.75" customHeight="1">
       <c r="D154" s="11"/>
@@ -9996,7 +9817,6 @@
       <c r="AY154" s="11"/>
       <c r="AZ154" s="11"/>
       <c r="BA154" s="11"/>
-      <c r="BB154" s="11"/>
     </row>
     <row r="155" ht="15.75" customHeight="1">
       <c r="D155" s="11"/>
@@ -10049,7 +9869,6 @@
       <c r="AY155" s="11"/>
       <c r="AZ155" s="11"/>
       <c r="BA155" s="11"/>
-      <c r="BB155" s="11"/>
     </row>
     <row r="156" ht="15.75" customHeight="1">
       <c r="D156" s="11"/>
@@ -10102,7 +9921,6 @@
       <c r="AY156" s="11"/>
       <c r="AZ156" s="11"/>
       <c r="BA156" s="11"/>
-      <c r="BB156" s="11"/>
     </row>
     <row r="157" ht="15.75" customHeight="1">
       <c r="D157" s="11"/>
@@ -10155,7 +9973,6 @@
       <c r="AY157" s="11"/>
       <c r="AZ157" s="11"/>
       <c r="BA157" s="11"/>
-      <c r="BB157" s="11"/>
     </row>
     <row r="158" ht="15.75" customHeight="1">
       <c r="D158" s="11"/>
@@ -10208,7 +10025,6 @@
       <c r="AY158" s="11"/>
       <c r="AZ158" s="11"/>
       <c r="BA158" s="11"/>
-      <c r="BB158" s="11"/>
     </row>
     <row r="159" ht="15.75" customHeight="1">
       <c r="D159" s="11"/>
@@ -10261,7 +10077,6 @@
       <c r="AY159" s="11"/>
       <c r="AZ159" s="11"/>
       <c r="BA159" s="11"/>
-      <c r="BB159" s="11"/>
     </row>
     <row r="160" ht="15.75" customHeight="1">
       <c r="D160" s="11"/>
@@ -10314,7 +10129,6 @@
       <c r="AY160" s="11"/>
       <c r="AZ160" s="11"/>
       <c r="BA160" s="11"/>
-      <c r="BB160" s="11"/>
     </row>
     <row r="161" ht="15.75" customHeight="1">
       <c r="D161" s="11"/>
@@ -10367,7 +10181,6 @@
       <c r="AY161" s="11"/>
       <c r="AZ161" s="11"/>
       <c r="BA161" s="11"/>
-      <c r="BB161" s="11"/>
     </row>
     <row r="162" ht="15.75" customHeight="1">
       <c r="D162" s="11"/>
@@ -10420,7 +10233,6 @@
       <c r="AY162" s="11"/>
       <c r="AZ162" s="11"/>
       <c r="BA162" s="11"/>
-      <c r="BB162" s="11"/>
     </row>
     <row r="163" ht="15.75" customHeight="1">
       <c r="D163" s="11"/>
@@ -10473,7 +10285,6 @@
       <c r="AY163" s="11"/>
       <c r="AZ163" s="11"/>
       <c r="BA163" s="11"/>
-      <c r="BB163" s="11"/>
     </row>
     <row r="164" ht="15.75" customHeight="1">
       <c r="D164" s="11"/>
@@ -10526,7 +10337,6 @@
       <c r="AY164" s="11"/>
       <c r="AZ164" s="11"/>
       <c r="BA164" s="11"/>
-      <c r="BB164" s="11"/>
     </row>
     <row r="165" ht="15.75" customHeight="1">
       <c r="D165" s="11"/>
@@ -10579,7 +10389,6 @@
       <c r="AY165" s="11"/>
       <c r="AZ165" s="11"/>
       <c r="BA165" s="11"/>
-      <c r="BB165" s="11"/>
     </row>
     <row r="166" ht="15.75" customHeight="1">
       <c r="D166" s="11"/>
@@ -10632,7 +10441,6 @@
       <c r="AY166" s="11"/>
       <c r="AZ166" s="11"/>
       <c r="BA166" s="11"/>
-      <c r="BB166" s="11"/>
     </row>
     <row r="167" ht="15.75" customHeight="1">
       <c r="D167" s="11"/>
@@ -10685,7 +10493,6 @@
       <c r="AY167" s="11"/>
       <c r="AZ167" s="11"/>
       <c r="BA167" s="11"/>
-      <c r="BB167" s="11"/>
     </row>
     <row r="168" ht="15.75" customHeight="1">
       <c r="D168" s="11"/>
@@ -10738,7 +10545,6 @@
       <c r="AY168" s="11"/>
       <c r="AZ168" s="11"/>
       <c r="BA168" s="11"/>
-      <c r="BB168" s="11"/>
     </row>
     <row r="169" ht="15.75" customHeight="1">
       <c r="D169" s="11"/>
@@ -10791,7 +10597,6 @@
       <c r="AY169" s="11"/>
       <c r="AZ169" s="11"/>
       <c r="BA169" s="11"/>
-      <c r="BB169" s="11"/>
     </row>
     <row r="170" ht="15.75" customHeight="1">
       <c r="D170" s="11"/>
@@ -10844,7 +10649,6 @@
       <c r="AY170" s="11"/>
       <c r="AZ170" s="11"/>
       <c r="BA170" s="11"/>
-      <c r="BB170" s="11"/>
     </row>
     <row r="171" ht="15.75" customHeight="1">
       <c r="D171" s="11"/>
@@ -10897,7 +10701,6 @@
       <c r="AY171" s="11"/>
       <c r="AZ171" s="11"/>
       <c r="BA171" s="11"/>
-      <c r="BB171" s="11"/>
     </row>
     <row r="172" ht="15.75" customHeight="1">
       <c r="D172" s="11"/>
@@ -10950,7 +10753,6 @@
       <c r="AY172" s="11"/>
       <c r="AZ172" s="11"/>
       <c r="BA172" s="11"/>
-      <c r="BB172" s="11"/>
     </row>
     <row r="173" ht="15.75" customHeight="1">
       <c r="D173" s="11"/>
@@ -11003,7 +10805,6 @@
       <c r="AY173" s="11"/>
       <c r="AZ173" s="11"/>
       <c r="BA173" s="11"/>
-      <c r="BB173" s="11"/>
     </row>
     <row r="174" ht="15.75" customHeight="1">
       <c r="D174" s="11"/>
@@ -11056,7 +10857,6 @@
       <c r="AY174" s="11"/>
       <c r="AZ174" s="11"/>
       <c r="BA174" s="11"/>
-      <c r="BB174" s="11"/>
     </row>
     <row r="175" ht="15.75" customHeight="1">
       <c r="D175" s="11"/>
@@ -11109,7 +10909,6 @@
       <c r="AY175" s="11"/>
       <c r="AZ175" s="11"/>
       <c r="BA175" s="11"/>
-      <c r="BB175" s="11"/>
     </row>
     <row r="176" ht="15.75" customHeight="1">
       <c r="D176" s="11"/>
@@ -11162,7 +10961,6 @@
       <c r="AY176" s="11"/>
       <c r="AZ176" s="11"/>
       <c r="BA176" s="11"/>
-      <c r="BB176" s="11"/>
     </row>
     <row r="177" ht="15.75" customHeight="1">
       <c r="D177" s="11"/>
@@ -11215,7 +11013,6 @@
       <c r="AY177" s="11"/>
       <c r="AZ177" s="11"/>
       <c r="BA177" s="11"/>
-      <c r="BB177" s="11"/>
     </row>
     <row r="178" ht="15.75" customHeight="1">
       <c r="D178" s="11"/>
@@ -11268,7 +11065,6 @@
       <c r="AY178" s="11"/>
       <c r="AZ178" s="11"/>
       <c r="BA178" s="11"/>
-      <c r="BB178" s="11"/>
     </row>
     <row r="179" ht="15.75" customHeight="1">
       <c r="D179" s="11"/>
@@ -11321,7 +11117,6 @@
       <c r="AY179" s="11"/>
       <c r="AZ179" s="11"/>
       <c r="BA179" s="11"/>
-      <c r="BB179" s="11"/>
     </row>
     <row r="180" ht="15.75" customHeight="1">
       <c r="D180" s="11"/>
@@ -11374,7 +11169,6 @@
       <c r="AY180" s="11"/>
       <c r="AZ180" s="11"/>
       <c r="BA180" s="11"/>
-      <c r="BB180" s="11"/>
     </row>
     <row r="181" ht="15.75" customHeight="1">
       <c r="D181" s="11"/>
@@ -11427,7 +11221,6 @@
       <c r="AY181" s="11"/>
       <c r="AZ181" s="11"/>
       <c r="BA181" s="11"/>
-      <c r="BB181" s="11"/>
     </row>
     <row r="182" ht="15.75" customHeight="1">
       <c r="D182" s="11"/>
@@ -11480,7 +11273,6 @@
       <c r="AY182" s="11"/>
       <c r="AZ182" s="11"/>
       <c r="BA182" s="11"/>
-      <c r="BB182" s="11"/>
     </row>
     <row r="183" ht="15.75" customHeight="1">
       <c r="D183" s="11"/>
@@ -11533,7 +11325,6 @@
       <c r="AY183" s="11"/>
       <c r="AZ183" s="11"/>
       <c r="BA183" s="11"/>
-      <c r="BB183" s="11"/>
     </row>
     <row r="184" ht="15.75" customHeight="1">
       <c r="D184" s="11"/>
@@ -11586,7 +11377,6 @@
       <c r="AY184" s="11"/>
       <c r="AZ184" s="11"/>
       <c r="BA184" s="11"/>
-      <c r="BB184" s="11"/>
     </row>
     <row r="185" ht="15.75" customHeight="1">
       <c r="D185" s="11"/>
@@ -11639,7 +11429,6 @@
       <c r="AY185" s="11"/>
       <c r="AZ185" s="11"/>
       <c r="BA185" s="11"/>
-      <c r="BB185" s="11"/>
     </row>
     <row r="186" ht="15.75" customHeight="1">
       <c r="D186" s="11"/>
@@ -11692,7 +11481,6 @@
       <c r="AY186" s="11"/>
       <c r="AZ186" s="11"/>
       <c r="BA186" s="11"/>
-      <c r="BB186" s="11"/>
     </row>
     <row r="187" ht="15.75" customHeight="1">
       <c r="D187" s="11"/>
@@ -11745,7 +11533,6 @@
       <c r="AY187" s="11"/>
       <c r="AZ187" s="11"/>
       <c r="BA187" s="11"/>
-      <c r="BB187" s="11"/>
     </row>
     <row r="188" ht="15.75" customHeight="1">
       <c r="D188" s="11"/>
@@ -11798,7 +11585,6 @@
       <c r="AY188" s="11"/>
       <c r="AZ188" s="11"/>
       <c r="BA188" s="11"/>
-      <c r="BB188" s="11"/>
     </row>
     <row r="189" ht="15.75" customHeight="1">
       <c r="D189" s="11"/>
@@ -11851,7 +11637,6 @@
       <c r="AY189" s="11"/>
       <c r="AZ189" s="11"/>
       <c r="BA189" s="11"/>
-      <c r="BB189" s="11"/>
     </row>
     <row r="190" ht="15.75" customHeight="1">
       <c r="D190" s="11"/>
@@ -11904,7 +11689,6 @@
       <c r="AY190" s="11"/>
       <c r="AZ190" s="11"/>
       <c r="BA190" s="11"/>
-      <c r="BB190" s="11"/>
     </row>
     <row r="191" ht="15.75" customHeight="1">
       <c r="D191" s="11"/>
@@ -11957,7 +11741,6 @@
       <c r="AY191" s="11"/>
       <c r="AZ191" s="11"/>
       <c r="BA191" s="11"/>
-      <c r="BB191" s="11"/>
     </row>
     <row r="192" ht="15.75" customHeight="1">
       <c r="D192" s="11"/>
@@ -12010,7 +11793,6 @@
       <c r="AY192" s="11"/>
       <c r="AZ192" s="11"/>
       <c r="BA192" s="11"/>
-      <c r="BB192" s="11"/>
     </row>
     <row r="193" ht="15.75" customHeight="1">
       <c r="D193" s="11"/>
@@ -12063,7 +11845,6 @@
       <c r="AY193" s="11"/>
       <c r="AZ193" s="11"/>
       <c r="BA193" s="11"/>
-      <c r="BB193" s="11"/>
     </row>
     <row r="194" ht="15.75" customHeight="1">
       <c r="D194" s="11"/>
@@ -12116,7 +11897,6 @@
       <c r="AY194" s="11"/>
       <c r="AZ194" s="11"/>
       <c r="BA194" s="11"/>
-      <c r="BB194" s="11"/>
     </row>
     <row r="195" ht="15.75" customHeight="1">
       <c r="D195" s="11"/>
@@ -12169,7 +11949,6 @@
       <c r="AY195" s="11"/>
       <c r="AZ195" s="11"/>
       <c r="BA195" s="11"/>
-      <c r="BB195" s="11"/>
     </row>
     <row r="196" ht="15.75" customHeight="1">
       <c r="D196" s="11"/>
@@ -12222,7 +12001,6 @@
       <c r="AY196" s="11"/>
       <c r="AZ196" s="11"/>
       <c r="BA196" s="11"/>
-      <c r="BB196" s="11"/>
     </row>
     <row r="197" ht="15.75" customHeight="1">
       <c r="D197" s="11"/>
@@ -12275,7 +12053,6 @@
       <c r="AY197" s="11"/>
       <c r="AZ197" s="11"/>
       <c r="BA197" s="11"/>
-      <c r="BB197" s="11"/>
     </row>
     <row r="198" ht="15.75" customHeight="1">
       <c r="D198" s="11"/>
@@ -12328,7 +12105,6 @@
       <c r="AY198" s="11"/>
       <c r="AZ198" s="11"/>
       <c r="BA198" s="11"/>
-      <c r="BB198" s="11"/>
     </row>
     <row r="199" ht="15.75" customHeight="1">
       <c r="D199" s="11"/>
@@ -12381,7 +12157,6 @@
       <c r="AY199" s="11"/>
       <c r="AZ199" s="11"/>
       <c r="BA199" s="11"/>
-      <c r="BB199" s="11"/>
     </row>
     <row r="200" ht="15.75" customHeight="1">
       <c r="D200" s="11"/>
@@ -12434,7 +12209,6 @@
       <c r="AY200" s="11"/>
       <c r="AZ200" s="11"/>
       <c r="BA200" s="11"/>
-      <c r="BB200" s="11"/>
     </row>
     <row r="201" ht="15.75" customHeight="1">
       <c r="D201" s="11"/>
@@ -12487,7 +12261,6 @@
       <c r="AY201" s="11"/>
       <c r="AZ201" s="11"/>
       <c r="BA201" s="11"/>
-      <c r="BB201" s="11"/>
     </row>
     <row r="202" ht="15.75" customHeight="1">
       <c r="D202" s="11"/>
@@ -12540,7 +12313,6 @@
       <c r="AY202" s="11"/>
       <c r="AZ202" s="11"/>
       <c r="BA202" s="11"/>
-      <c r="BB202" s="11"/>
     </row>
     <row r="203" ht="15.75" customHeight="1">
       <c r="D203" s="11"/>
@@ -12593,7 +12365,6 @@
       <c r="AY203" s="11"/>
       <c r="AZ203" s="11"/>
       <c r="BA203" s="11"/>
-      <c r="BB203" s="11"/>
     </row>
     <row r="204" ht="15.75" customHeight="1">
       <c r="D204" s="11"/>
@@ -12646,7 +12417,6 @@
       <c r="AY204" s="11"/>
       <c r="AZ204" s="11"/>
       <c r="BA204" s="11"/>
-      <c r="BB204" s="11"/>
     </row>
     <row r="205" ht="15.75" customHeight="1">
       <c r="D205" s="11"/>
@@ -12699,7 +12469,6 @@
       <c r="AY205" s="11"/>
       <c r="AZ205" s="11"/>
       <c r="BA205" s="11"/>
-      <c r="BB205" s="11"/>
     </row>
     <row r="206" ht="15.75" customHeight="1">
       <c r="D206" s="11"/>
@@ -12752,7 +12521,6 @@
       <c r="AY206" s="11"/>
       <c r="AZ206" s="11"/>
       <c r="BA206" s="11"/>
-      <c r="BB206" s="11"/>
     </row>
     <row r="207" ht="15.75" customHeight="1">
       <c r="D207" s="11"/>
@@ -12805,7 +12573,6 @@
       <c r="AY207" s="11"/>
       <c r="AZ207" s="11"/>
       <c r="BA207" s="11"/>
-      <c r="BB207" s="11"/>
     </row>
     <row r="208" ht="15.75" customHeight="1">
       <c r="D208" s="11"/>
@@ -12858,7 +12625,6 @@
       <c r="AY208" s="11"/>
       <c r="AZ208" s="11"/>
       <c r="BA208" s="11"/>
-      <c r="BB208" s="11"/>
     </row>
     <row r="209" ht="15.75" customHeight="1">
       <c r="D209" s="11"/>
@@ -12911,7 +12677,6 @@
       <c r="AY209" s="11"/>
       <c r="AZ209" s="11"/>
       <c r="BA209" s="11"/>
-      <c r="BB209" s="11"/>
     </row>
     <row r="210" ht="15.75" customHeight="1">
       <c r="D210" s="11"/>
@@ -12964,7 +12729,6 @@
       <c r="AY210" s="11"/>
       <c r="AZ210" s="11"/>
       <c r="BA210" s="11"/>
-      <c r="BB210" s="11"/>
     </row>
     <row r="211" ht="15.75" customHeight="1">
       <c r="D211" s="11"/>
@@ -13017,7 +12781,6 @@
       <c r="AY211" s="11"/>
       <c r="AZ211" s="11"/>
       <c r="BA211" s="11"/>
-      <c r="BB211" s="11"/>
     </row>
     <row r="212" ht="15.75" customHeight="1">
       <c r="D212" s="11"/>
@@ -13070,7 +12833,6 @@
       <c r="AY212" s="11"/>
       <c r="AZ212" s="11"/>
       <c r="BA212" s="11"/>
-      <c r="BB212" s="11"/>
     </row>
     <row r="213" ht="15.75" customHeight="1">
       <c r="D213" s="11"/>
@@ -13123,7 +12885,6 @@
       <c r="AY213" s="11"/>
       <c r="AZ213" s="11"/>
       <c r="BA213" s="11"/>
-      <c r="BB213" s="11"/>
     </row>
     <row r="214" ht="15.75" customHeight="1">
       <c r="D214" s="11"/>
@@ -13176,7 +12937,6 @@
       <c r="AY214" s="11"/>
       <c r="AZ214" s="11"/>
       <c r="BA214" s="11"/>
-      <c r="BB214" s="11"/>
     </row>
     <row r="215" ht="15.75" customHeight="1">
       <c r="D215" s="11"/>
@@ -13229,7 +12989,6 @@
       <c r="AY215" s="11"/>
       <c r="AZ215" s="11"/>
       <c r="BA215" s="11"/>
-      <c r="BB215" s="11"/>
     </row>
     <row r="216" ht="15.75" customHeight="1">
       <c r="D216" s="11"/>
@@ -13282,7 +13041,6 @@
       <c r="AY216" s="11"/>
       <c r="AZ216" s="11"/>
       <c r="BA216" s="11"/>
-      <c r="BB216" s="11"/>
     </row>
     <row r="217" ht="15.75" customHeight="1">
       <c r="D217" s="11"/>
@@ -13335,7 +13093,6 @@
       <c r="AY217" s="11"/>
       <c r="AZ217" s="11"/>
       <c r="BA217" s="11"/>
-      <c r="BB217" s="11"/>
     </row>
     <row r="218" ht="15.75" customHeight="1">
       <c r="D218" s="11"/>
@@ -13388,7 +13145,6 @@
       <c r="AY218" s="11"/>
       <c r="AZ218" s="11"/>
       <c r="BA218" s="11"/>
-      <c r="BB218" s="11"/>
     </row>
     <row r="219" ht="15.75" customHeight="1">
       <c r="D219" s="11"/>
@@ -13441,7 +13197,6 @@
       <c r="AY219" s="11"/>
       <c r="AZ219" s="11"/>
       <c r="BA219" s="11"/>
-      <c r="BB219" s="11"/>
     </row>
     <row r="220" ht="15.75" customHeight="1">
       <c r="D220" s="11"/>
@@ -13494,7 +13249,6 @@
       <c r="AY220" s="11"/>
       <c r="AZ220" s="11"/>
       <c r="BA220" s="11"/>
-      <c r="BB220" s="11"/>
     </row>
     <row r="221" ht="15.75" customHeight="1"/>
     <row r="222" ht="15.75" customHeight="1"/>
@@ -14278,12 +14032,12 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:G1"/>
     <mergeCell ref="H1:N1"/>
-    <mergeCell ref="X1:BB1"/>
     <mergeCell ref="O1:P1"/>
     <mergeCell ref="Q1:W1"/>
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="X1:BA1"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>